<commit_message>
Website update 2026-06-19 00:44:18
</commit_message>
<xml_diff>
--- a/gitrepo/build/source/lasvillasweb.xlsx
+++ b/gitrepo/build/source/lasvillasweb.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B2CB268-73F3-4E29-B355-9E52CCADEAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Homepage" sheetId="1" r:id="rId1"/>
@@ -785,7 +785,7 @@
     <row r="5" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="12">
         <f ca="1">NOW()</f>
-        <v>46190.999475694443</v>
+        <v>46192.023207175924</v>
       </c>
       <c r="B5" s="12"/>
     </row>

</xml_diff>